<commit_message>
ksoft - 8280 - 06/03/2026 - Hora: 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft_old/_bakas/Papeis DP E FF.xlsx
+++ b/ksoft_old/_bakas/Papeis DP E FF.xlsx
@@ -6224,13 +6224,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80C82D26-83B9-4453-A9C2-659BEFF341B4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B74695EE-1940-43BD-AF58-2BDF06E872DC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A4C0E5F-8055-464E-A3F2-1A2757090B9D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4DE4BA8-B927-49EE-82C5-DD3B6538A470}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20DD7D8E-D330-4B7F-9D1A-3F59CC82D136}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24CC7E53-1838-4C86-A9D6-8AD81D640F93}"/>
 </file>
</xml_diff>

<commit_message>
ksoft - 8280 - 13/03/2026 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft_old/_bakas/Papeis DP E FF.xlsx
+++ b/ksoft_old/_bakas/Papeis DP E FF.xlsx
@@ -6224,13 +6224,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B74695EE-1940-43BD-AF58-2BDF06E872DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99318C3E-E9DE-410F-B73E-106663221A87}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4DE4BA8-B927-49EE-82C5-DD3B6538A470}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40AB7C64-A8AC-4C98-8FC3-AABD3C0BF8A9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24CC7E53-1838-4C86-A9D6-8AD81D640F93}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C86EF901-3C90-4ED2-8B77-FD4FA3FDD2D5}"/>
 </file>
</xml_diff>

<commit_message>
ksoft - 8280 - 23/03/2026 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft_old/_bakas/Papeis DP E FF.xlsx
+++ b/ksoft_old/_bakas/Papeis DP E FF.xlsx
@@ -6224,13 +6224,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99318C3E-E9DE-410F-B73E-106663221A87}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80C82D26-83B9-4453-A9C2-659BEFF341B4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40AB7C64-A8AC-4C98-8FC3-AABD3C0BF8A9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A4C0E5F-8055-464E-A3F2-1A2757090B9D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C86EF901-3C90-4ED2-8B77-FD4FA3FDD2D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20DD7D8E-D330-4B7F-9D1A-3F59CC82D136}"/>
 </file>
</xml_diff>